<commit_message>
Add HATSUTAKA fuel exhaustion theory from HAWKBILL's patrol report
</commit_message>
<xml_diff>
--- a/patrolReports/Cobia_inferred_positions.xlsx
+++ b/patrolReports/Cobia_inferred_positions.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -58,11 +58,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,7 +489,7 @@
       <c r="D2" t="n">
         <v>-14</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>16249</v>
       </c>
       <c r="F2" t="n">
@@ -515,7 +517,7 @@
       <c r="D3" t="n">
         <v>-12</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <v>16253</v>
       </c>
       <c r="F3" t="n">
@@ -543,7 +545,7 @@
       <c r="D4" t="n">
         <v>-10</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>16259</v>
       </c>
       <c r="F4" t="n">
@@ -571,7 +573,7 @@
       <c r="D5" t="n">
         <v>-9</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>16262</v>
       </c>
       <c r="F5" t="n">
@@ -599,7 +601,7 @@
       <c r="D6" t="n">
         <v>-9</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>16265</v>
       </c>
       <c r="F6" t="n">
@@ -627,7 +629,7 @@
       <c r="D7" t="n">
         <v>-9</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>16266</v>
       </c>
       <c r="F7" t="n">
@@ -655,7 +657,7 @@
       <c r="D8" t="n">
         <v>-9</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>16267</v>
       </c>
       <c r="F8" t="n">
@@ -683,7 +685,7 @@
       <c r="D9" t="n">
         <v>-9</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>16271</v>
       </c>
       <c r="F9" t="n">
@@ -711,7 +713,7 @@
       <c r="D10" t="n">
         <v>-9</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>16271</v>
       </c>
       <c r="F10" t="n">
@@ -739,7 +741,7 @@
       <c r="D11" t="n">
         <v>-9</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="3" t="n">
         <v>16273</v>
       </c>
       <c r="F11" t="n">
@@ -767,7 +769,7 @@
       <c r="D12" t="n">
         <v>-9</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="3" t="n">
         <v>16273</v>
       </c>
       <c r="F12" t="n">
@@ -795,7 +797,7 @@
       <c r="D13" t="n">
         <v>-9</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="3" t="n">
         <v>16289</v>
       </c>
       <c r="F13" t="n">
@@ -823,7 +825,7 @@
       <c r="D14" t="n">
         <v>-12</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="3" t="n">
         <v>16298</v>
       </c>
       <c r="F14" t="n">
@@ -851,7 +853,7 @@
       <c r="D15" t="n">
         <v>-12</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="3" t="n">
         <v>16321</v>
       </c>
       <c r="F15" t="n">
@@ -879,7 +881,7 @@
       <c r="D16" t="n">
         <v>-12</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="3" t="n">
         <v>16324</v>
       </c>
       <c r="F16" t="n">
@@ -907,7 +909,7 @@
       <c r="D17" t="n">
         <v>-11</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="3" t="n">
         <v>16328</v>
       </c>
       <c r="F17" t="n">
@@ -935,7 +937,7 @@
       <c r="D18" t="n">
         <v>-9</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="3" t="n">
         <v>16349</v>
       </c>
       <c r="F18" t="n">
@@ -963,7 +965,7 @@
       <c r="D19" t="n">
         <v>-9</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="3" t="n">
         <v>16350</v>
       </c>
       <c r="F19" t="n">
@@ -991,7 +993,7 @@
       <c r="D20" t="n">
         <v>-9</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="3" t="n">
         <v>16364</v>
       </c>
       <c r="F20" t="n">
@@ -1019,7 +1021,7 @@
       <c r="D21" t="n">
         <v>-9</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="3" t="n">
         <v>16366</v>
       </c>
       <c r="F21" t="n">
@@ -1047,7 +1049,7 @@
       <c r="D22" t="n">
         <v>-9</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="3" t="n">
         <v>16372</v>
       </c>
       <c r="F22" t="n">
@@ -1075,7 +1077,7 @@
       <c r="D23" t="n">
         <v>-9</v>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="E23" s="3" t="n">
         <v>16375</v>
       </c>
       <c r="F23" t="n">
@@ -1103,7 +1105,7 @@
       <c r="D24" t="n">
         <v>-9</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="3" t="n">
         <v>16378</v>
       </c>
       <c r="F24" t="n">
@@ -1131,7 +1133,7 @@
       <c r="D25" t="n">
         <v>-9</v>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="E25" s="3" t="n">
         <v>16381</v>
       </c>
       <c r="F25" t="n">
@@ -1159,7 +1161,7 @@
       <c r="D26" t="n">
         <v>-9</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="3" t="n">
         <v>16406</v>
       </c>
       <c r="F26" t="n">
@@ -1187,7 +1189,7 @@
       <c r="D27" t="n">
         <v>-9</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="3" t="n">
         <v>16408</v>
       </c>
       <c r="F27" t="n">
@@ -1215,7 +1217,7 @@
       <c r="D28" t="n">
         <v>-9</v>
       </c>
-      <c r="E28" s="2" t="n">
+      <c r="E28" s="3" t="n">
         <v>16409</v>
       </c>
       <c r="F28" t="n">
@@ -1243,7 +1245,7 @@
       <c r="D29" t="n">
         <v>-9</v>
       </c>
-      <c r="E29" s="2" t="n">
+      <c r="E29" s="3" t="n">
         <v>16415</v>
       </c>
       <c r="F29" t="n">
@@ -1271,7 +1273,7 @@
       <c r="D30" t="n">
         <v>-9</v>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="E30" s="3" t="n">
         <v>16417</v>
       </c>
       <c r="F30" t="n">
@@ -1291,26 +1293,26 @@
         <v>3</v>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C31" t="n">
-        <v>1352</v>
+        <v>330</v>
       </c>
       <c r="D31" t="n">
         <v>-9</v>
       </c>
-      <c r="E31" s="2" t="n">
-        <v>16451</v>
+      <c r="E31" s="4" t="n">
+        <v>16445</v>
       </c>
       <c r="F31" t="n">
-        <v>5.852</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>103.317</v>
+        <v>115.22</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Torpedo Attack #1</t>
+          <t>Commodore Reef reconnaissance</t>
         </is>
       </c>
     </row>
@@ -1319,26 +1321,26 @@
         <v>3</v>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C32" t="n">
-        <v>300</v>
+        <v>457</v>
       </c>
       <c r="D32" t="n">
         <v>-9</v>
       </c>
-      <c r="E32" s="2" t="n">
-        <v>16454</v>
+      <c r="E32" s="4" t="n">
+        <v>16445</v>
       </c>
       <c r="F32" t="n">
-        <v>-3.02</v>
+        <v>8.064064999999999</v>
       </c>
       <c r="G32" t="n">
-        <v>109.138</v>
+        <v>114.733344</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Cleared Karimata Strait</t>
+          <t>Investigator Shoal reconnaissance</t>
         </is>
       </c>
     </row>
@@ -1347,26 +1349,26 @@
         <v>3</v>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C33" t="n">
-        <v>1555</v>
+        <v>730</v>
       </c>
       <c r="D33" t="n">
         <v>-9</v>
       </c>
-      <c r="E33" s="2" t="n">
-        <v>16454</v>
+      <c r="E33" s="4" t="n">
+        <v>16445</v>
       </c>
       <c r="F33" t="n">
-        <v>-5.428</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G33" t="n">
-        <v>112.505</v>
+        <v>114.16</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Sighted Bawean Island</t>
+          <t>Cornwallis South Reef reconnaissance</t>
         </is>
       </c>
     </row>
@@ -1375,26 +1377,26 @@
         <v>3</v>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C34" t="n">
-        <v>2250</v>
+        <v>848</v>
       </c>
       <c r="D34" t="n">
         <v>-9</v>
       </c>
-      <c r="E34" s="2" t="n">
-        <v>16454</v>
+      <c r="E34" s="4" t="n">
+        <v>16445</v>
       </c>
       <c r="F34" t="n">
-        <v>-5.86</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G34" t="n">
-        <v>114.282</v>
+        <v>114.08</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Sighted Masalembu Island</t>
+          <t>Alison Reef reconnaissance</t>
         </is>
       </c>
     </row>
@@ -1403,26 +1405,26 @@
         <v>3</v>
       </c>
       <c r="B35" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C35" t="n">
-        <v>1255</v>
+        <v>1725</v>
       </c>
       <c r="D35" t="n">
         <v>-9</v>
       </c>
-      <c r="E35" s="2" t="n">
-        <v>16455</v>
+      <c r="E35" s="4" t="n">
+        <v>16445</v>
       </c>
       <c r="F35" t="n">
-        <v>-7.503</v>
+        <v>7.57</v>
       </c>
       <c r="G35" t="n">
-        <v>116.048</v>
+        <v>111.65</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Sighted Lombok Island</t>
+          <t>Rifleman Bank reconnaissance</t>
         </is>
       </c>
     </row>
@@ -1431,26 +1433,26 @@
         <v>3</v>
       </c>
       <c r="B36" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>258</v>
+        <v>1352</v>
       </c>
       <c r="D36" t="n">
         <v>-9</v>
       </c>
-      <c r="E36" s="2" t="n">
-        <v>16458</v>
+      <c r="E36" s="3" t="n">
+        <v>16451</v>
       </c>
       <c r="F36" t="n">
-        <v>-22.219</v>
+        <v>5.852</v>
       </c>
       <c r="G36" t="n">
-        <v>114.119</v>
+        <v>103.317</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Refuel Exmouth Gulf</t>
+          <t>Torpedo Attack #1</t>
         </is>
       </c>
     </row>
@@ -1459,26 +1461,26 @@
         <v>3</v>
       </c>
       <c r="B37" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C37" t="n">
-        <v>1915</v>
+        <v>300</v>
       </c>
       <c r="D37" t="n">
         <v>-9</v>
       </c>
-      <c r="E37" s="2" t="n">
-        <v>16458</v>
+      <c r="E37" s="3" t="n">
+        <v>16454</v>
       </c>
       <c r="F37" t="n">
-        <v>-21.772</v>
+        <v>-3.02</v>
       </c>
       <c r="G37" t="n">
-        <v>114.299</v>
+        <v>109.138</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Cleared Exmouth Gulf</t>
+          <t>Cleared Karimata Strait</t>
         </is>
       </c>
     </row>
@@ -1487,26 +1489,26 @@
         <v>3</v>
       </c>
       <c r="B38" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C38" t="n">
-        <v>130</v>
+        <v>1555</v>
       </c>
       <c r="D38" t="n">
         <v>-9</v>
       </c>
-      <c r="E38" s="2" t="n">
-        <v>16459</v>
+      <c r="E38" s="3" t="n">
+        <v>16454</v>
       </c>
       <c r="F38" t="n">
-        <v>-21.787</v>
+        <v>-5.428</v>
       </c>
       <c r="G38" t="n">
-        <v>111.5</v>
+        <v>112.505</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Interpolated</t>
+          <t>Sighted Bawean Island</t>
         </is>
       </c>
     </row>
@@ -1515,166 +1517,166 @@
         <v>3</v>
       </c>
       <c r="B39" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C39" t="n">
-        <v>800</v>
+        <v>2250</v>
       </c>
       <c r="D39" t="n">
         <v>-9</v>
       </c>
-      <c r="E39" s="2" t="n">
-        <v>16461</v>
+      <c r="E39" s="3" t="n">
+        <v>16454</v>
       </c>
       <c r="F39" t="n">
-        <v>-32.05</v>
+        <v>-5.86</v>
       </c>
       <c r="G39" t="n">
-        <v>115.742</v>
+        <v>114.282</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Freemantle sub base</t>
+          <t>Sighted Masalembu Island</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C40" t="n">
-        <v>1320</v>
+        <v>1255</v>
       </c>
       <c r="D40" t="n">
         <v>-9</v>
       </c>
-      <c r="E40" s="2" t="n">
-        <v>16486</v>
+      <c r="E40" s="3" t="n">
+        <v>16455</v>
       </c>
       <c r="F40" t="n">
-        <v>-32.05</v>
+        <v>-7.503</v>
       </c>
       <c r="G40" t="n">
-        <v>115.742</v>
+        <v>116.048</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Freemantle sub base</t>
+          <t>Sighted Lombok Island</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B41" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C41" t="n">
-        <v>1630</v>
+        <v>258</v>
       </c>
       <c r="D41" t="n">
         <v>-9</v>
       </c>
-      <c r="E41" s="2" t="n">
-        <v>16494</v>
+      <c r="E41" s="3" t="n">
+        <v>16458</v>
       </c>
       <c r="F41" t="n">
-        <v>-6.117</v>
+        <v>-22.219</v>
       </c>
       <c r="G41" t="n">
-        <v>114.1</v>
+        <v>114.119</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Gun Attack No. 1</t>
+          <t>Refuel Exmouth Gulf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B42" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C42" t="n">
-        <v>1815</v>
+        <v>1915</v>
       </c>
       <c r="D42" t="n">
         <v>-9</v>
       </c>
-      <c r="E42" s="2" t="n">
-        <v>16494</v>
+      <c r="E42" s="3" t="n">
+        <v>16458</v>
       </c>
       <c r="F42" t="n">
-        <v>-6.12</v>
+        <v>-21.772</v>
       </c>
       <c r="G42" t="n">
-        <v>114.11</v>
+        <v>114.299</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Gun Attack No. 2</t>
+          <t>Cleared Exmouth Gulf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B43" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C43" t="n">
-        <v>941</v>
+        <v>130</v>
       </c>
       <c r="D43" t="n">
         <v>-9</v>
       </c>
-      <c r="E43" s="2" t="n">
-        <v>16500</v>
+      <c r="E43" s="3" t="n">
+        <v>16459</v>
       </c>
       <c r="F43" t="n">
-        <v>-32.05</v>
+        <v>-21.787</v>
       </c>
       <c r="G43" t="n">
-        <v>115.742</v>
+        <v>111.5</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Freemantle sub base</t>
+          <t>Interpolated</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B44" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C44" t="n">
-        <v>649</v>
+        <v>800</v>
       </c>
       <c r="D44" t="n">
         <v>-9</v>
       </c>
-      <c r="E44" s="2" t="n">
-        <v>16507</v>
+      <c r="E44" s="3" t="n">
+        <v>16461</v>
       </c>
       <c r="F44" t="n">
-        <v>-21.9</v>
+        <v>-32.05</v>
       </c>
       <c r="G44" t="n">
-        <v>114.15</v>
+        <v>115.742</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Exmouth Gulf refueling</t>
+          <t>Freemantle sub base</t>
         </is>
       </c>
     </row>
@@ -1683,26 +1685,26 @@
         <v>4</v>
       </c>
       <c r="B45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>1433</v>
+        <v>1320</v>
       </c>
       <c r="D45" t="n">
         <v>-9</v>
       </c>
-      <c r="E45" s="2" t="n">
-        <v>16510</v>
+      <c r="E45" s="3" t="n">
+        <v>16486</v>
       </c>
       <c r="F45" t="n">
-        <v>-5.667</v>
+        <v>-32.05</v>
       </c>
       <c r="G45" t="n">
-        <v>114.233</v>
+        <v>115.742</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Torpedo Attack No. 1</t>
+          <t>Freemantle sub base</t>
         </is>
       </c>
     </row>
@@ -1711,26 +1713,26 @@
         <v>4</v>
       </c>
       <c r="B46" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C46" t="n">
-        <v>238</v>
+        <v>1630</v>
       </c>
       <c r="D46" t="n">
         <v>-9</v>
       </c>
-      <c r="E46" s="2" t="n">
-        <v>16526</v>
+      <c r="E46" s="3" t="n">
+        <v>16494</v>
       </c>
       <c r="F46" t="n">
-        <v>11.833</v>
+        <v>-6.117</v>
       </c>
       <c r="G46" t="n">
-        <v>109.35</v>
+        <v>114.1</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Torpedo Attack No. 2</t>
+          <t>Gun Attack No. 1</t>
         </is>
       </c>
     </row>
@@ -1739,134 +1741,134 @@
         <v>4</v>
       </c>
       <c r="B47" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C47" t="n">
-        <v>1200</v>
+        <v>1815</v>
       </c>
       <c r="D47" t="n">
         <v>-9</v>
       </c>
-      <c r="E47" s="2" t="n">
-        <v>16542</v>
+      <c r="E47" s="3" t="n">
+        <v>16494</v>
       </c>
       <c r="F47" t="n">
-        <v>14.82</v>
+        <v>-6.12</v>
       </c>
       <c r="G47" t="n">
-        <v>120.211</v>
+        <v>114.11</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Subic Bay Base</t>
+          <t>Gun Attack No. 2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C48" t="n">
-        <v>1407</v>
+        <v>941</v>
       </c>
       <c r="D48" t="n">
         <v>-9</v>
       </c>
-      <c r="E48" s="2" t="n">
-        <v>16566</v>
+      <c r="E48" s="3" t="n">
+        <v>16500</v>
       </c>
       <c r="F48" t="n">
-        <v>14.82</v>
+        <v>-32.05</v>
       </c>
       <c r="G48" t="n">
-        <v>120.211</v>
+        <v>115.742</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Subic Bay Base</t>
+          <t>Freemantle sub base</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
+        <v>4</v>
+      </c>
+      <c r="B49" t="n">
         <v>5</v>
       </c>
-      <c r="B49" t="n">
-        <v>2</v>
-      </c>
       <c r="C49" t="n">
-        <v>737</v>
+        <v>649</v>
       </c>
       <c r="D49" t="n">
         <v>-9</v>
       </c>
-      <c r="E49" s="2" t="n">
-        <v>16571</v>
+      <c r="E49" s="3" t="n">
+        <v>16507</v>
       </c>
       <c r="F49" t="n">
-        <v>9.583</v>
+        <v>-21.9</v>
       </c>
       <c r="G49" t="n">
-        <v>101.733</v>
+        <v>114.15</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Torpedo Attack No. 1</t>
+          <t>Exmouth Gulf refueling</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B50" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C50" t="n">
-        <v>1909</v>
+        <v>1433</v>
       </c>
       <c r="D50" t="n">
         <v>-9</v>
       </c>
-      <c r="E50" s="2" t="n">
-        <v>16587</v>
+      <c r="E50" s="3" t="n">
+        <v>16510</v>
       </c>
       <c r="F50" t="n">
-        <v>10.2</v>
+        <v>-5.667</v>
       </c>
       <c r="G50" t="n">
-        <v>99.233</v>
+        <v>114.233</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Gun Attack No. 1</t>
+          <t>Torpedo Attack No. 1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B51" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C51" t="n">
-        <v>410</v>
+        <v>238</v>
       </c>
       <c r="D51" t="n">
         <v>-9</v>
       </c>
-      <c r="E51" s="2" t="n">
-        <v>16596</v>
+      <c r="E51" s="3" t="n">
+        <v>16526</v>
       </c>
       <c r="F51" t="n">
-        <v>8.933</v>
+        <v>11.833</v>
       </c>
       <c r="G51" t="n">
-        <v>105.633</v>
+        <v>109.35</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -1876,29 +1878,29 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B52" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C52" t="n">
-        <v>438</v>
+        <v>1200</v>
       </c>
       <c r="D52" t="n">
         <v>-9</v>
       </c>
-      <c r="E52" s="2" t="n">
-        <v>16596</v>
+      <c r="E52" s="3" t="n">
+        <v>16542</v>
       </c>
       <c r="F52" t="n">
-        <v>8.93</v>
+        <v>14.82</v>
       </c>
       <c r="G52" t="n">
-        <v>105.63</v>
+        <v>120.211</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Torpedo Attack No. 3</t>
+          <t>Subic Bay Base</t>
         </is>
       </c>
     </row>
@@ -1907,26 +1909,26 @@
         <v>5</v>
       </c>
       <c r="B53" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C53" t="n">
-        <v>518</v>
+        <v>1407</v>
       </c>
       <c r="D53" t="n">
         <v>-9</v>
       </c>
-      <c r="E53" s="2" t="n">
-        <v>16596</v>
+      <c r="E53" s="3" t="n">
+        <v>16566</v>
       </c>
       <c r="F53" t="n">
-        <v>8.927</v>
+        <v>14.82</v>
       </c>
       <c r="G53" t="n">
-        <v>105.636</v>
+        <v>120.211</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Torpedo Attack No. 4</t>
+          <t>Subic Bay Base</t>
         </is>
       </c>
     </row>
@@ -1935,26 +1937,26 @@
         <v>5</v>
       </c>
       <c r="B54" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C54" t="n">
-        <v>637</v>
+        <v>737</v>
       </c>
       <c r="D54" t="n">
         <v>-9</v>
       </c>
-      <c r="E54" s="2" t="n">
-        <v>16596</v>
+      <c r="E54" s="3" t="n">
+        <v>16571</v>
       </c>
       <c r="F54" t="n">
-        <v>8.936</v>
+        <v>9.583</v>
       </c>
       <c r="G54" t="n">
-        <v>105.639</v>
+        <v>101.733</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Torpedo Attack No. 5</t>
+          <t>Torpedo Attack No. 1</t>
         </is>
       </c>
     </row>
@@ -1963,26 +1965,26 @@
         <v>5</v>
       </c>
       <c r="B55" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C55" t="n">
-        <v>842</v>
+        <v>1909</v>
       </c>
       <c r="D55" t="n">
         <v>-9</v>
       </c>
-      <c r="E55" s="2" t="n">
-        <v>16603</v>
+      <c r="E55" s="3" t="n">
+        <v>16587</v>
       </c>
       <c r="F55" t="n">
-        <v>-21.64</v>
+        <v>10.2</v>
       </c>
       <c r="G55" t="n">
-        <v>115.11</v>
+        <v>99.233</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Onslow Jetty refueling</t>
+          <t>Gun Attack No. 1</t>
         </is>
       </c>
     </row>
@@ -1991,162 +1993,166 @@
         <v>5</v>
       </c>
       <c r="B56" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C56" t="n">
-        <v>1200</v>
+        <v>410</v>
       </c>
       <c r="D56" t="n">
         <v>-9</v>
       </c>
-      <c r="E56" s="2" t="n">
-        <v>16606</v>
+      <c r="E56" s="3" t="n">
+        <v>16596</v>
       </c>
       <c r="F56" t="n">
-        <v>-32.05</v>
+        <v>8.933</v>
       </c>
       <c r="G56" t="n">
-        <v>115.742</v>
+        <v>105.633</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Freemantle sub base</t>
+          <t>Torpedo Attack No. 2</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>438</v>
       </c>
       <c r="D57" t="n">
         <v>-9</v>
       </c>
-      <c r="E57" s="2" t="n">
-        <v>16637</v>
+      <c r="E57" s="3" t="n">
+        <v>16596</v>
       </c>
       <c r="F57" t="n">
-        <v>-32.05</v>
+        <v>8.93</v>
       </c>
       <c r="G57" t="n">
-        <v>115.742</v>
+        <v>105.63</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Freemantle sub base</t>
+          <t>Torpedo Attack No. 3</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
+        <v>5</v>
+      </c>
+      <c r="B58" t="n">
         <v>6</v>
       </c>
-      <c r="B58" t="n">
-        <v>2</v>
-      </c>
       <c r="C58" t="n">
-        <v>200</v>
+        <v>518</v>
       </c>
       <c r="D58" t="n">
         <v>-9</v>
       </c>
-      <c r="E58" s="2" t="n">
-        <v>16642</v>
+      <c r="E58" s="3" t="n">
+        <v>16596</v>
       </c>
       <c r="F58" t="n">
-        <v>-8.822699999999999</v>
+        <v>8.927</v>
       </c>
       <c r="G58" t="n">
-        <v>114.49</v>
+        <v>105.636</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Blambangan Pensinsula</t>
+          <t>Torpedo Attack No. 4</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B59" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C59" t="n">
-        <v>330</v>
+        <v>637</v>
       </c>
       <c r="D59" t="n">
         <v>-9</v>
       </c>
-      <c r="E59" s="2" t="n">
-        <v>16642</v>
+      <c r="E59" s="3" t="n">
+        <v>16596</v>
       </c>
       <c r="F59" t="n">
-        <v>-8.659000000000001</v>
+        <v>8.936</v>
       </c>
       <c r="G59" t="n">
-        <v>114.222</v>
+        <v>105.639</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Grajagan Bay</t>
+          <t>Torpedo Attack No. 5</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B60" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C60" t="n">
-        <v>2010</v>
+        <v>842</v>
       </c>
       <c r="D60" t="n">
         <v>-9</v>
       </c>
-      <c r="E60" s="2" t="n">
-        <v>16643</v>
+      <c r="E60" s="3" t="n">
+        <v>16603</v>
       </c>
       <c r="F60" t="n">
-        <v>-7.418</v>
+        <v>-21.64</v>
       </c>
       <c r="G60" t="n">
-        <v>105.357</v>
-      </c>
-      <c r="H60" t="inlineStr"/>
+        <v>115.11</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Onslow Jetty refueling</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B61" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C61" t="n">
-        <v>740</v>
+        <v>1200</v>
       </c>
       <c r="D61" t="n">
         <v>-9</v>
       </c>
-      <c r="E61" s="2" t="n">
-        <v>16644</v>
+      <c r="E61" s="3" t="n">
+        <v>16606</v>
       </c>
       <c r="F61" t="n">
-        <v>-6.485</v>
+        <v>-32.05</v>
       </c>
       <c r="G61" t="n">
-        <v>104.936</v>
+        <v>115.742</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Submerged off 3rd point</t>
+          <t>Freemantle sub base</t>
         </is>
       </c>
     </row>
@@ -2155,26 +2161,26 @@
         <v>6</v>
       </c>
       <c r="B62" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C62" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="D62" t="n">
         <v>-9</v>
       </c>
-      <c r="E62" s="2" t="n">
-        <v>16645</v>
+      <c r="E62" s="3" t="n">
+        <v>16637</v>
       </c>
       <c r="F62" t="n">
-        <v>-5.934</v>
+        <v>-32.05</v>
       </c>
       <c r="G62" t="n">
-        <v>105.8</v>
+        <v>115.742</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Sangiang Island (Thwartway)</t>
+          <t>Freemantle sub base</t>
         </is>
       </c>
     </row>
@@ -2183,26 +2189,26 @@
         <v>6</v>
       </c>
       <c r="B63" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C63" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D63" t="n">
         <v>-9</v>
       </c>
-      <c r="E63" s="2" t="n">
-        <v>16645</v>
+      <c r="E63" s="3" t="n">
+        <v>16642</v>
       </c>
       <c r="F63" t="n">
-        <v>-6.1</v>
+        <v>-8.822699999999999</v>
       </c>
       <c r="G63" t="n">
-        <v>105.85</v>
+        <v>114.49</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Landed 4 Javanese commandos on the west coast of Java</t>
+          <t>Blambangan Pensinsula</t>
         </is>
       </c>
     </row>
@@ -2211,26 +2217,26 @@
         <v>6</v>
       </c>
       <c r="B64" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C64" t="n">
-        <v>213</v>
+        <v>330</v>
       </c>
       <c r="D64" t="n">
         <v>-9</v>
       </c>
-      <c r="E64" s="2" t="n">
-        <v>16647</v>
+      <c r="E64" s="3" t="n">
+        <v>16642</v>
       </c>
       <c r="F64" t="n">
-        <v>-2.34</v>
+        <v>-8.659000000000001</v>
       </c>
       <c r="G64" t="n">
-        <v>109.05</v>
+        <v>114.222</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Karimata Island</t>
+          <t>Grajagan Bay</t>
         </is>
       </c>
     </row>
@@ -2239,27 +2245,22 @@
         <v>6</v>
       </c>
       <c r="B65" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C65" t="n">
-        <v>810</v>
+        <v>2010</v>
       </c>
       <c r="D65" t="n">
         <v>-9</v>
       </c>
-      <c r="E65" s="2" t="n">
-        <v>16648</v>
+      <c r="E65" s="3" t="n">
+        <v>16643</v>
       </c>
       <c r="F65" t="n">
-        <v>4.22</v>
+        <v>-7.418</v>
       </c>
       <c r="G65" t="n">
-        <v>107.22</v>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>Great Natoena Island</t>
-        </is>
+        <v>105.357</v>
       </c>
     </row>
     <row r="66">
@@ -2267,26 +2268,26 @@
         <v>6</v>
       </c>
       <c r="B66" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C66" t="n">
-        <v>1005</v>
+        <v>740</v>
       </c>
       <c r="D66" t="n">
         <v>-9</v>
       </c>
-      <c r="E66" s="2" t="n">
-        <v>16654</v>
+      <c r="E66" s="3" t="n">
+        <v>16644</v>
       </c>
       <c r="F66" t="n">
-        <v>14.82</v>
+        <v>-6.485</v>
       </c>
       <c r="G66" t="n">
-        <v>120.211</v>
+        <v>104.936</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Subic Bay Base</t>
+          <t>Submerged off 3rd point</t>
         </is>
       </c>
     </row>
@@ -2295,98 +2296,110 @@
         <v>6</v>
       </c>
       <c r="B67" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C67" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="D67" t="n">
         <v>-9</v>
       </c>
-      <c r="E67" s="2" t="n">
-        <v>16660</v>
+      <c r="E67" s="3" t="n">
+        <v>16645</v>
       </c>
       <c r="F67" t="n">
-        <v>21.4</v>
+        <v>-5.934</v>
       </c>
       <c r="G67" t="n">
-        <v>120.5</v>
-      </c>
-      <c r="H67" t="inlineStr"/>
+        <v>105.8</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Sangiang Island (Thwartway)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
         <v>6</v>
       </c>
       <c r="B68" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C68" t="n">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="D68" t="n">
         <v>-9</v>
       </c>
-      <c r="E68" s="2" t="n">
-        <v>16661</v>
+      <c r="E68" s="3" t="n">
+        <v>16645</v>
       </c>
       <c r="F68" t="n">
-        <v>21.4</v>
+        <v>-6.1</v>
       </c>
       <c r="G68" t="n">
-        <v>123.5</v>
-      </c>
-      <c r="H68" t="inlineStr"/>
+        <v>105.85</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Landed 4 Javanese commandos on the west coast of Java</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
         <v>6</v>
       </c>
       <c r="B69" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C69" t="n">
-        <v>2000</v>
+        <v>213</v>
       </c>
       <c r="D69" t="n">
         <v>-9</v>
       </c>
-      <c r="E69" s="2" t="n">
-        <v>16661</v>
+      <c r="E69" s="3" t="n">
+        <v>16647</v>
       </c>
       <c r="F69" t="n">
-        <v>21.4</v>
+        <v>-2.34</v>
       </c>
       <c r="G69" t="n">
-        <v>123</v>
-      </c>
-      <c r="H69" t="inlineStr"/>
+        <v>109.05</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Karimata Island</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
         <v>6</v>
       </c>
       <c r="B70" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C70" t="n">
-        <v>2050</v>
+        <v>810</v>
       </c>
       <c r="D70" t="n">
         <v>-9</v>
       </c>
-      <c r="E70" s="2" t="n">
-        <v>16663</v>
+      <c r="E70" s="3" t="n">
+        <v>16648</v>
       </c>
       <c r="F70" t="n">
-        <v>22.33</v>
+        <v>4.22</v>
       </c>
       <c r="G70" t="n">
-        <v>120.17</v>
+        <v>107.22</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Log entry: "Japan has accepted the terms offered her (unofficially)"</t>
+          <t>Great Natoena Island</t>
         </is>
       </c>
     </row>
@@ -2395,26 +2408,26 @@
         <v>6</v>
       </c>
       <c r="B71" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C71" t="n">
-        <v>1500</v>
+        <v>1005</v>
       </c>
       <c r="D71" t="n">
         <v>-9</v>
       </c>
-      <c r="E71" s="2" t="n">
-        <v>16667</v>
+      <c r="E71" s="3" t="n">
+        <v>16654</v>
       </c>
       <c r="F71" t="n">
-        <v>23.23</v>
+        <v>14.82</v>
       </c>
       <c r="G71" t="n">
-        <v>125.49</v>
+        <v>120.211</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Rendezvoused with ICEFISH, CROAKER, RAY, and JACK, all enroute to Saipan.</t>
+          <t>Subic Bay Base</t>
         </is>
       </c>
     </row>
@@ -2423,24 +2436,149 @@
         <v>6</v>
       </c>
       <c r="B72" t="n">
+        <v>11</v>
+      </c>
+      <c r="C72" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D72" t="n">
+        <v>-9</v>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>16660</v>
+      </c>
+      <c r="F72" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="G72" t="n">
+        <v>120.5</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>6</v>
+      </c>
+      <c r="B73" t="n">
+        <v>12</v>
+      </c>
+      <c r="C73" t="n">
+        <v>600</v>
+      </c>
+      <c r="D73" t="n">
+        <v>-9</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>16661</v>
+      </c>
+      <c r="F73" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="G73" t="n">
+        <v>123.5</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>6</v>
+      </c>
+      <c r="B74" t="n">
+        <v>13</v>
+      </c>
+      <c r="C74" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D74" t="n">
+        <v>-9</v>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>16661</v>
+      </c>
+      <c r="F74" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="G74" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>6</v>
+      </c>
+      <c r="B75" t="n">
+        <v>14</v>
+      </c>
+      <c r="C75" t="n">
+        <v>2050</v>
+      </c>
+      <c r="D75" t="n">
+        <v>-9</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>16663</v>
+      </c>
+      <c r="F75" t="n">
+        <v>22.33</v>
+      </c>
+      <c r="G75" t="n">
+        <v>120.17</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Log entry: "Japan has accepted the terms offered her (unofficially)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>6</v>
+      </c>
+      <c r="B76" t="n">
+        <v>15</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D76" t="n">
+        <v>-9</v>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>16667</v>
+      </c>
+      <c r="F76" t="n">
+        <v>23.23</v>
+      </c>
+      <c r="G76" t="n">
+        <v>125.49</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Rendezvoused with ICEFISH, CROAKER, RAY, and JACK, all enroute to Saipan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>6</v>
+      </c>
+      <c r="B77" t="n">
         <v>16</v>
       </c>
-      <c r="C72" t="n">
+      <c r="C77" t="n">
         <v>1200</v>
       </c>
-      <c r="D72" t="n">
+      <c r="D77" t="n">
         <v>-10</v>
       </c>
-      <c r="E72" s="2" t="n">
+      <c r="E77" s="3" t="n">
         <v>16671</v>
       </c>
-      <c r="F72" t="n">
+      <c r="F77" t="n">
         <v>15.222</v>
       </c>
-      <c r="G72" t="n">
+      <c r="G77" t="n">
         <v>145.728</v>
       </c>
-      <c r="H72" t="inlineStr">
+      <c r="H77" t="inlineStr">
         <is>
           <t>Saipan Naval Advance Base</t>
         </is>

</xml_diff>